<commit_message>
Add Key Account Plant data
</commit_message>
<xml_diff>
--- a/Dataset.sample.xlsx
+++ b/Dataset.sample.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yongj\Projects\apac-visualizer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BAD106C8-1454-42F7-9570-8827D6F337A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{68F9569D-ABB0-474B-8F9D-49EB368F01C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2595" yWindow="2595" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,8 @@
     <sheet name="Region Vertical Overview" sheetId="1" r:id="rId1"/>
     <sheet name="Dealer List" sheetId="2" r:id="rId2"/>
     <sheet name="Dealer Customer List" sheetId="4" r:id="rId3"/>
-    <sheet name="Priority Target List" sheetId="3" r:id="rId4"/>
+    <sheet name="Key Account List" sheetId="5" r:id="rId4"/>
+    <sheet name="Priority Target List" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="40">
   <si>
     <t>F&amp;B</t>
   </si>
@@ -178,6 +179,10 @@
   </si>
   <si>
     <t>ID</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Account Name</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -842,6 +847,68 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6A2162D-637D-4E8B-B1DC-2D121E22F7F5}">
+  <dimension ref="A1:O1"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="9" style="3"/>
+    <col min="6" max="7" width="9" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Q1"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>

</xml_diff>